<commit_message>
Implementación de Seguridad OWASP y buenas practicas de seguridad
</commit_message>
<xml_diff>
--- a/datos_prueba/pedidos_demo.xlsx
+++ b/datos_prueba/pedidos_demo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,20 +424,40 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>cliente_origen</t>
+          <t>razon_social_cliente</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>ruc_cliente</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>direccion_destino</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>nombre_destinatario</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>telefono_destinatario</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dni_destinatario</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>peso_kg</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>volumen_m3</t>
         </is>
@@ -451,18 +471,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tienda ACME</t>
+          <t>Tienda ACME SAC</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>20100000001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Av. Brasil 1234, San Miguel, Lima, Peru</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>987654321</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>45678912</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
         <v>2.5</v>
       </c>
-      <c r="E2" t="n">
+      <c r="I2" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -474,18 +514,38 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Botica Fast</t>
+          <t>Botica Fast EIRL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>20100000002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Av. La Marina 2500, San Miguel, Lima, Peru</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Maria Lopez</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>912345678</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>10293847</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="n">
+      <c r="I3" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -497,18 +557,38 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Libreria Sur</t>
+          <t>Libreria Sur SAC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>20100000003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Av. Universitaria 1801, San Miguel, Lima, Peru</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Carlos Ruiz</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>998877665</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>73645123</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
         <v>3.2</v>
       </c>
-      <c r="E4" t="n">
+      <c r="I4" t="n">
         <v>0.03</v>
       </c>
     </row>
@@ -520,18 +600,38 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Moda XYZ</t>
+          <t>Moda XYZ SAC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>20100000004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Av. Larco 345, Miraflores, Lima, Peru</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Ana Torres</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>955443322</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>60718293</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
         <v>0.8</v>
       </c>
-      <c r="E5" t="n">
+      <c r="I5" t="n">
         <v>0.005</v>
       </c>
     </row>
@@ -543,18 +643,38 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TechStore</t>
+          <t>TechStore SAC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>20100000005</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Av. Arequipa 4500, Miraflores, Lima, Peru</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Luis Diaz</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>933221100</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>80910111</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
         <v>1.5</v>
       </c>
-      <c r="E6" t="n">
+      <c r="I6" t="n">
         <v>0.02</v>
       </c>
     </row>

</xml_diff>